<commit_message>
Gap register Rev 7: resolve G-49/G-50/G-52 from call answers
Decommission gate: 7-day monitored hold, authorization signed by Kyle
Mandersfield. Post-Exchange recipient management: WMP-owned processes,
no Essendis PowerShell runbooks. Operations and support: out of
engagement scope (WMP decides alerting; Azure subscription available;
the design's Log Analytics wording is cleaned up under G-03). 13 open
(11 High / 2 Medium), 51 resolved.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9SFx2c7BjowTfENYrpiQo
</commit_message>
<xml_diff>
--- a/deliverables/WMP/WMP__Solution_Design_Gap_Register__20260825.xlsx
+++ b/deliverables/WMP/WMP__Solution_Design_Gap_Register__20260825.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Resolved Decisions" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Gap Register'!$A$1:$K$17</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Resolved Decisions'!$A$1:$E$49</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Gap Register'!$A$1:$K$14</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Resolved Decisions'!$A$1:$E$52</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,12 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="329">
   <si>
     <t xml:space="preserve">WMP Solution Design — Inputs &amp; Decisions Gap Register</t>
   </si>
   <si>
-    <t xml:space="preserve">Rev 6 — 8/25/2026: WMP status dispositions applied; the 16 remaining rows are phrased as short, call-ready questions.</t>
+    <t xml:space="preserve">Rev 7 — 8/25/2026: call answers applied (decommission gate, post-Exchange ownership, operations scope). 13 call-ready rows remain.</t>
   </si>
   <si>
     <t xml:space="preserve">Wisconsin Metal Parts — Microsoft GCC High Migration (CMMC 2.0 Level 2)  |  Prepared by Essendis</t>
@@ -403,58 +403,6 @@
   </si>
   <si>
     <t xml:space="preserve">New section: Endpoint Configuration &gt; On-Premises Resource Access; Device Migration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G-49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The pre-decommission gate lists what must be true but not how it is proven. "No applications or services still authenticating" and "no SMTP relay dependencies" are assertions with no monitoring method, no observation period, and no evidence artifact; the monitored-hold duration is left as "until confirmed idle".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decommission is one-way past the point of hybrid removal; a relay client discovered afterwards means mail loss with only a server backup as the recovery route.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How long is the monitored hold before Exchange removal — 7, 14, or 30 days?
-Who at WMP signs the decommission authorisation?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migration Design &gt; Pre-Decommission Validation Gate; Monitored Hold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G-50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The document states that after decommission, recipient management moves to "Entra ID Connect and PowerShell against Active Directory attributes" with no Exchange management server retained — but no runbook, tooling, or skills transfer is defined for that day-2 reality.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creating a mailbox, adding a proxy address, or building a distribution list from raw AD attributes is error-prone and unfamiliar; WMP will need to do it in week one after handoff and there is nothing written to follow.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Who at WMP will manage mailboxes/aliases/groups after Exchange is gone? (Essendis provides the PowerShell runbook and training.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migration Design &gt; Hybrid Configuration and Directory Services; As-Configured document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G-52</t>
-  </si>
-  <si>
-    <t xml:space="preserve">There is no monitoring or alerting design. The only alert in the document is break-glass sign-in detection "via Log Analytics in Azure" — a service that is out of scope — and nothing routes Defender, Intune, identity, or service-health alerts to a human.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMMC AU.L2-3.3.1/3.3.5 and IR.L2-3.6.1 expect logs to be reviewed and incidents detected; alerts nobody receives are not a detective control, and the break-glass alert as designed cannot be built.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An Azure subscription exists: use Log Analytics for break-glass/audit alerting, or stay M365-native?
-Who receives security alerts (Defender, Intune, Entra) — which mailbox or Teams channel?
-What log-review cadence and owner should we document?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">There is an available Azure subscription, need to make decision whether log analytics is required.
-WMP (8/25): an Azure subscription is available — decide whether Log Analytics is used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline Security &gt; Emergency Accounts; new "Monitoring &amp; Alerting" section</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -908,6 +856,30 @@
     <t xml:space="preserve">Windows device inventory by site/type is collected by WMP during pre-migration device preparation (WBS 7.1.1); Windows 11/TPM exceptions are handled wave-by-wave; servers remain out of scope (G-28).</t>
   </si>
   <si>
+    <t xml:space="preserve">G-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The pre-decommission gate lists what must be true but not how it is proven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WMP (8/25, via chat): 7-day monitored hold; Kyle Mandersfield signs the decommission authorization.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design update: the pre-removal monitored hold is 7 days and the decommission authorization is signed by Kyle Mandersfield (WMP). Essendis defines the residual-connection evidence check within that window.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The document states that after decommission, recipient management moves to "Entra ID Connect and PowerShell against Active Directory attributes" with no Exchange management server retained — but no runbook, tooling, or skills transfer is defined for that day-2 reality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WMP (8/25, via chat): Essendis is not providing runbooks for PowerShell-based management; WMP owns the processes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design update: post-decommission recipient management is WMP-owned. The design notes management continues via Entra Connect/PowerShell with no Essendis runbook deliverable.</t>
+  </si>
+  <si>
     <t xml:space="preserve">G-51</t>
   </si>
   <si>
@@ -918,6 +890,18 @@
   </si>
   <si>
     <t xml:space="preserve">Support model set: hypercare runs one week post-migration with a 2-hour response objective; requests via email and Teams; WMP handles user-facing support thereafter. Essendis documents this in the Communications/support section.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">There is no monitoring or alerting design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WMP (8/25, via chat): Operations and support are out of scope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope decision: monitoring, alerting, and log-review design are out of engagement scope — WMP decides (an Azure subscription exists if Log Analytics is wanted). Essendis's remaining action is the G-03 cleanup: reword the design's break-glass 'Log Analytics in Azure' reference to reflect WMP-owned alerting.</t>
   </si>
   <si>
     <t xml:space="preserve">G-53</t>
@@ -1264,24 +1248,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1289,7 +1277,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1297,19 +1285,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1326,6 +1314,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1633,187 +1625,187 @@
   <dimension ref="B2:F25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="s">
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="8" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B18)</f>
         <v>2</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F18" s="9" t="n">
+      <c r="F18" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!J:J,"High")</f>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B19)</f>
         <v>2</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F19" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!J:J,"Medium")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C20" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B20)</f>
         <v>3</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="11" t="n">
+      <c r="F20" s="12" t="n">
         <f aca="false">COUNTA('Gap Register'!A:A)-1</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B21)</f>
         <v>1</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="11" t="n">
+      <c r="F21" s="12" t="n">
         <f aca="false">COUNTA('Resolved Decisions'!A:A)-1</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B22)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B23)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="9" t="n">
+      <c r="C24" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B24)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="8" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="9" t="n">
+      <c r="C25" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B25)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1840,602 +1832,540 @@
   <dimension ref="A1:K17"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="8"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="13" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+    <row r="2" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13" t="s">
+      <c r="G2" s="14"/>
+      <c r="H2" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+    <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+    <row r="4" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="K4" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J5" s="14" t="s">
+      <c r="J5" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="K5" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+    <row r="6" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13" t="s">
+      <c r="G6" s="14"/>
+      <c r="H6" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J6" s="14" t="s">
+      <c r="J6" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="K6" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+    <row r="7" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13" t="s">
+      <c r="G7" s="14"/>
+      <c r="H7" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="J7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="K7" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+    <row r="8" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="15" t="s">
+      <c r="J8" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K8" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
+    <row r="9" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="J9" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="K9" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+    <row r="10" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J10" s="14" t="s">
+      <c r="J10" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="K10" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+    <row r="11" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="J11" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="K11" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
+    <row r="12" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13" t="s">
+      <c r="G12" s="14"/>
+      <c r="H12" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J12" s="14" t="s">
+      <c r="J12" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K12" s="13" t="s">
+      <c r="K12" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+    <row r="13" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="G13" s="13" t="s">
+      <c r="G13" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="H13" s="13" t="s">
+      <c r="H13" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="I13" s="13" t="s">
+      <c r="I13" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="J13" s="14" t="s">
+      <c r="J13" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K13" s="13" t="s">
+      <c r="K13" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+    <row r="14" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13" t="s">
+      <c r="G14" s="14"/>
+      <c r="H14" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="I14" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="J14" s="14" t="s">
+      <c r="J14" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="K14" s="13" t="s">
+      <c r="K14" s="14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="J15" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K15" s="13" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="I16" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="J16" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="K16" s="13" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="I17" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="J17" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K17" s="13" t="s">
-        <v>42</v>
-      </c>
+    <row r="15" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+    </row>
+    <row r="16" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+    </row>
+    <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K17"/>
+  <autoFilter ref="A1:K14"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2452,850 +2382,901 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="B5" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="D5" s="14" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B2" s="13" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B21" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="C17" s="13" t="s">
+      <c r="C21" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D21" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E21" s="14" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+    <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="B18" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="C18" s="13" t="s">
+      <c r="B22" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D22" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E22" s="14" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+    <row r="23" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="B19" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="13" t="s">
+      <c r="B23" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D23" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E23" s="14" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+    <row r="24" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="13" t="s">
+      <c r="B24" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D24" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E24" s="14" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
+    <row r="25" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
         <v>215</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B25" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C25" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D25" s="14" t="s">
         <v>217</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E25" s="14" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+    <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B26" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C26" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D26" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E26" s="14" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
+    <row r="27" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>223</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B27" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C27" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D27" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E27" s="14" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+    <row r="28" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
         <v>227</v>
       </c>
-      <c r="B24" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="13" t="s">
+      <c r="B28" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D28" s="14" t="s">
         <v>229</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E28" s="14" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+    <row r="29" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="B25" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="13" t="s">
+      <c r="B29" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D29" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E29" s="14" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="13" t="s">
+      <c r="B30" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>236</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D30" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E30" s="14" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
+    <row r="31" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="B27" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="13" t="s">
+      <c r="B31" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D31" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E31" s="14" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
+    <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="B28" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="13" t="s">
+      <c r="B32" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D32" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E32" s="14" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
+    <row r="33" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C29" s="13" t="s">
+      <c r="B33" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D33" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E33" s="14" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="s">
         <v>251</v>
       </c>
-      <c r="B30" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C30" s="13" t="s">
+      <c r="B34" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D34" s="14" t="s">
         <v>253</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E34" s="14" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
+    <row r="35" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B35" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C35" s="14" t="s">
         <v>256</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D35" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E35" s="14" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
+    <row r="36" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="B32" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C32" s="13" t="s">
+      <c r="B36" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D36" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="E36" s="14" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
+    <row r="37" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="s">
         <v>263</v>
       </c>
-      <c r="B33" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C33" s="13" t="s">
+      <c r="B37" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D37" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="E33" s="13" t="s">
+      <c r="E37" s="14" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
         <v>267</v>
       </c>
-      <c r="B34" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C34" s="13" t="s">
+      <c r="B38" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C38" s="14" t="s">
         <v>268</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D38" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="E38" s="14" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="s">
         <v>271</v>
       </c>
-      <c r="B35" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C35" s="13" t="s">
+      <c r="B39" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>272</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="D39" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="E39" s="14" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14" t="s">
         <v>275</v>
       </c>
-      <c r="B36" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C36" s="13" t="s">
+      <c r="B40" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D40" s="14" t="s">
         <v>277</v>
       </c>
-      <c r="E36" s="13" t="s">
+      <c r="E40" s="14" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="s">
+    <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="B37" s="13" t="s">
+      <c r="B41" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C41" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="D41" s="14" t="s">
         <v>281</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E41" s="14" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
+    <row r="42" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B42" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C42" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D42" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E42" s="14" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
+    <row r="43" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B43" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C39" s="13" t="s">
+      <c r="C43" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="D39" s="13" t="s">
+      <c r="D43" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="E39" s="13" t="s">
+      <c r="E43" s="14" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="s">
+    <row r="44" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="B40" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C40" s="13" t="s">
+      <c r="B44" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="C44" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="E40" s="13" t="s">
+      <c r="D44" s="14" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
+      <c r="E44" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="B41" s="13" t="s">
+    </row>
+    <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="C41" s="13" t="s">
+      <c r="B45" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="C45" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="D41" s="13" t="s">
+      <c r="D45" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E45" s="14" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
+    <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="B42" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="C42" s="13" t="s">
+      <c r="B46" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="C46" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D46" s="14" t="s">
         <v>302</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E46" s="14" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="s">
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="B43" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="C43" s="13" t="s">
+      <c r="B47" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="C47" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="D43" s="13" t="s">
+      <c r="D47" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="E47" s="14" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
+    <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
         <v>308</v>
       </c>
-      <c r="B44" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="C44" s="13" t="s">
+      <c r="B48" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="C48" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D48" s="14" t="s">
         <v>310</v>
       </c>
-      <c r="E44" s="13" t="s">
+      <c r="E48" s="14" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="13" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="s">
         <v>312</v>
       </c>
-      <c r="B45" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="C45" s="13" t="s">
+      <c r="B49" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="C49" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D49" s="14" t="s">
         <v>314</v>
       </c>
-      <c r="E45" s="13" t="s">
+      <c r="E49" s="14" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="13" t="s">
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="s">
         <v>316</v>
       </c>
-      <c r="B46" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="C46" s="13" t="s">
+      <c r="B50" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="C50" s="14" t="s">
         <v>317</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D50" s="14" t="s">
         <v>318</v>
       </c>
-      <c r="E46" s="13" t="s">
+      <c r="E50" s="14" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="13" t="s">
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
         <v>320</v>
       </c>
-      <c r="B47" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="C47" s="13" t="s">
+      <c r="B51" s="14" t="s">
         <v>321</v>
       </c>
-      <c r="D47" s="13" t="s">
+      <c r="C51" s="14" t="s">
         <v>322</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="D51" s="14" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13" t="s">
+      <c r="E51" s="14" t="s">
         <v>324</v>
       </c>
-      <c r="B48" s="13" t="s">
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="C48" s="13" t="s">
+      <c r="B52" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="C52" s="14" t="s">
         <v>326</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="D52" s="14" t="s">
         <v>327</v>
       </c>
-      <c r="E48" s="13" t="s">
+      <c r="E52" s="14" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="B49" s="13" t="s">
-        <v>325</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>330</v>
-      </c>
-      <c r="D49" s="13" t="s">
-        <v>331</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>332</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E49"/>
+  <autoFilter ref="A1:E52"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>